<commit_message>
Corrección de errores y mejoras.
</commit_message>
<xml_diff>
--- a/Output/Excel/Mascotas.xlsx
+++ b/Output/Excel/Mascotas.xlsx
@@ -37,25 +37,139 @@
     <x:t>Enlace</x:t>
   </x:si>
   <x:si>
-    <x:t>VICKY</x:t>
+    <x:t>ZALAMERO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Macho</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Burro </x:t>
+  </x:si>
+  <x:si>
+    <x:t>5 años  y   7 meses</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Mediano</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> ZALAMERO es nuestro niño bonito, es tan noble que nos tiene enamorados. Cuando lo recogimos venía tan desnutrido que teníamos que no pudiera sobrevivir.  No deberíamos permitir que ningún animal muriera de hambre, sin embargo, la realidad es que como protectora no podemos hacernos cargo de todos los que nos necesitan.  Aunque a Zalamero ya no le va a faltar quien cuide de él. Desde que siente la barriga llena se le ve contento y con ganas de cariños. Es muy tierno.  Necesitamos madrinas y padrinos que nos ayuden. </x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://arcadenoe.org/ficha-580</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OREJOTAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>5 años  y   9 meses</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> OREJOTAS es el burrito más cariñoso y sociable que hemos conocido. Es tan bueno como bonito.  La subida del precio del grano y el heno ha provocado que algunos dueños hayan tenido que ceder a sus equinos.  Nosotros nos hemos hecho cargo de OREJOTAS porque lo necesitaba pero buscamos padrinos que nos ayuden hasta que encontremos una buena familia que le adopte.  </x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://arcadenoe.org/ficha-573</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MELOCOTÓN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Poni</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9 años  y   11 meses</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Pequeño</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> Nos llegó un aviso de que había entrado un poni en la perrera de Sevilla, aunque nos sorprendió luego aprendimos que por desgracia no es un caso raro. Los equinos también acaban malviviendo en la perrera municipal, y si para los perros es un mal sitio para ellos es aún peor. Nos pusimos manos a la obra y conseguimos sacarlo de allí, ahora vive en nuestro refugio, es muy feliz y nos está enseñando a ser una protectora también de ponis. Es nuestro chico mimado por lo que no se dará en adopción si no es para vivir en mejores condiciones de las que ya está.  Melocontón no es una herramienta de trabajo, no es un muñeco de juguete, es un ser vivo que necesita cariño y capaz de darlo.  Si crees que en tu vida hay hueco para él, no dudes en escribirnos. </x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://arcadenoe.org/ficha-519</x:t>
+  </x:si>
+  <x:si>
+    <x:t>JUEVES (JUEVITA)</x:t>
   </x:si>
   <x:si>
     <x:t>Hembra</x:t>
   </x:si>
   <x:si>
-    <x:t>Naranja</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9 años  y   8 meses</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Mediano</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> Vicky es asustadiza. Tiene un problema nervioso que hace que cada vez que se asusta da vueltas en circulo. Le encantan las latitas de comida húmeda y dormir en sitios donde se siente protegida.   Me rescataron de la calle, enferma y muuuy asustada. </x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://arcadenoe.org/ficha-641</x:t>
+    <x:t xml:space="preserve"> Fue rescatada un jueves, un caluroso jueves de julio, solita y llorando desolada. Esta gatita tricolor es una aventurera. Le gusta cotillear y subirse donde puede para buscar tus cariños. Se lleva bien con los otros gatos y le encanta que le den mimos.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://arcadenoe.org/ficha-600</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DUQUESA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8 años  y   9 meses</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> Ajustándose a su nombre, esta gatita es digna de la realeza. Duquesa es una gata elegante y apacible, le encanta relajarse al sol. No obstante, no te dirá que no si te apetece darle cariño.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://arcadenoe.org/ficha-599</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MELANIA (BIGOTINA)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9 años  y   7 meses</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> Muy asustadiza y poco sociable.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://arcadenoe.org/ficha-636</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OCARINA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12 años</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> </x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://arcadenoe.org/ficha-632</x:t>
+  </x:si>
+  <x:si>
+    <x:t>JULIA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8 años  y   1 mes</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> Esta gatita fue rescatada de un contenedor por un voluntario ...  Esta pequeñina es muy especial, curiosa y juguetona, aunque un poco desconfiada. Le encanta explorar y jugar con su compañero Blacky. Con los voluntarios necesita confianza para dejarse acariciar y mostrar su lado más cariñoso.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://arcadenoe.org/ficha-601</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INGRID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Europeo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8 años  y   11 meses</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> Soy una gatita ronroneadora, súper mimosa y muy dulce.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://arcadenoe.org/ficha-355</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CANDELA2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10 años  y   8 meses</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://arcadenoe.org/ficha-629</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -457,7 +571,7 @@
     </x:row>
     <x:row r="3" spans="1:7">
       <x:c r="A3" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>8</x:v>
@@ -466,200 +580,182 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:7">
       <x:c r="A4" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:7">
       <x:c r="A5" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="G5" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:7">
       <x:c r="A6" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G6" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:7">
       <x:c r="A7" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C7" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="F7" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="G7" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:7">
       <x:c r="A8" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C8" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E8" s="0" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="F8" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="G8" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>39</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:7">
       <x:c r="A9" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C9" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="E9" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F9" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="G9" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>43</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:7">
       <x:c r="A10" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="D10" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="E10" s="0" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="F10" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="G10" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>48</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:7">
       <x:c r="A11" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C11" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D11" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="E11" s="0" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="F11" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="G11" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>51</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>